<commit_message>
Add schedule extension Add possibility to filter by ytm Add possibility to order by closing date Add possibility to peek selected number of rows Add possibility to print rows
</commit_message>
<xml_diff>
--- a/src/main/resources/secondary-market/secondary-market-example.xlsx
+++ b/src/main/resources/secondary-market/secondary-market-example.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2274" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2274" uniqueCount="546">
   <si>
     <t>Country</t>
   </si>
@@ -190,139 +190,142 @@
     <t>169.54</t>
   </si>
   <si>
+    <t>88321644-01</t>
+  </si>
+  <si>
+    <t>19.03.2020</t>
+  </si>
+  <si>
+    <t>83.98</t>
+  </si>
+  <si>
+    <t>83.90</t>
+  </si>
+  <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>8910655-01</t>
+  </si>
+  <si>
+    <t>15.11.2017</t>
+  </si>
+  <si>
+    <t>14.11.2019</t>
+  </si>
+  <si>
+    <t>Aasa</t>
+  </si>
+  <si>
+    <t>A-</t>
+  </si>
+  <si>
+    <t>9.00</t>
+  </si>
+  <si>
+    <t>9.0</t>
+  </si>
+  <si>
+    <t>66.50</t>
+  </si>
+  <si>
+    <t>0.0</t>
+  </si>
+  <si>
+    <t>8910302-01</t>
+  </si>
+  <si>
+    <t>01.12.2017</t>
+  </si>
+  <si>
+    <t>10.01.2020</t>
+  </si>
+  <si>
+    <t>42.44</t>
+  </si>
+  <si>
+    <t>9040152-01</t>
+  </si>
+  <si>
+    <t>20.12.2017</t>
+  </si>
+  <si>
+    <t>19.01.2020</t>
+  </si>
+  <si>
+    <t>68.51</t>
+  </si>
+  <si>
+    <t>11488954-01</t>
+  </si>
+  <si>
+    <t>20.02.2018</t>
+  </si>
+  <si>
+    <t>23.02.2020</t>
+  </si>
+  <si>
+    <t>73.71</t>
+  </si>
+  <si>
+    <t>11488958-01</t>
+  </si>
+  <si>
+    <t>23.02.2018</t>
+  </si>
+  <si>
+    <t>25.02.2020</t>
+  </si>
+  <si>
+    <t>68.99</t>
+  </si>
+  <si>
+    <t>5321615-01</t>
+  </si>
+  <si>
+    <t>10.03.2020</t>
+  </si>
+  <si>
+    <t>10.5</t>
+  </si>
+  <si>
+    <t>50.28</t>
+  </si>
+  <si>
+    <t>5321662-01</t>
+  </si>
+  <si>
+    <t>05.03.2020</t>
+  </si>
+  <si>
+    <t>11.0</t>
+  </si>
+  <si>
+    <t>38.89</t>
+  </si>
+  <si>
+    <t>5101389-01</t>
+  </si>
+  <si>
+    <t>05.09.2018</t>
+  </si>
+  <si>
+    <t>16.03.2020</t>
+  </si>
+  <si>
+    <t>1050.62</t>
+  </si>
+  <si>
+    <t>5341597-01</t>
+  </si>
+  <si>
+    <t>1235.47</t>
+  </si>
+  <si>
+    <t>100.50</t>
+  </si>
+  <si>
     <t>5321644-01</t>
-  </si>
-  <si>
-    <t>19.03.2020</t>
-  </si>
-  <si>
-    <t>83.98</t>
-  </si>
-  <si>
-    <t>83.90</t>
-  </si>
-  <si>
-    <t>EUR</t>
-  </si>
-  <si>
-    <t>8910655-01</t>
-  </si>
-  <si>
-    <t>15.11.2017</t>
-  </si>
-  <si>
-    <t>14.11.2019</t>
-  </si>
-  <si>
-    <t>Aasa</t>
-  </si>
-  <si>
-    <t>A-</t>
-  </si>
-  <si>
-    <t>9.00</t>
-  </si>
-  <si>
-    <t>9.0</t>
-  </si>
-  <si>
-    <t>66.50</t>
-  </si>
-  <si>
-    <t>0.0</t>
-  </si>
-  <si>
-    <t>8910302-01</t>
-  </si>
-  <si>
-    <t>01.12.2017</t>
-  </si>
-  <si>
-    <t>10.01.2020</t>
-  </si>
-  <si>
-    <t>42.44</t>
-  </si>
-  <si>
-    <t>9040152-01</t>
-  </si>
-  <si>
-    <t>20.12.2017</t>
-  </si>
-  <si>
-    <t>19.01.2020</t>
-  </si>
-  <si>
-    <t>68.51</t>
-  </si>
-  <si>
-    <t>11488954-01</t>
-  </si>
-  <si>
-    <t>20.02.2018</t>
-  </si>
-  <si>
-    <t>23.02.2020</t>
-  </si>
-  <si>
-    <t>73.71</t>
-  </si>
-  <si>
-    <t>11488958-01</t>
-  </si>
-  <si>
-    <t>23.02.2018</t>
-  </si>
-  <si>
-    <t>25.02.2020</t>
-  </si>
-  <si>
-    <t>68.99</t>
-  </si>
-  <si>
-    <t>5321615-01</t>
-  </si>
-  <si>
-    <t>10.03.2020</t>
-  </si>
-  <si>
-    <t>10.5</t>
-  </si>
-  <si>
-    <t>50.28</t>
-  </si>
-  <si>
-    <t>5321662-01</t>
-  </si>
-  <si>
-    <t>05.03.2020</t>
-  </si>
-  <si>
-    <t>11.0</t>
-  </si>
-  <si>
-    <t>38.89</t>
-  </si>
-  <si>
-    <t>5101389-01</t>
-  </si>
-  <si>
-    <t>05.09.2018</t>
-  </si>
-  <si>
-    <t>16.03.2020</t>
-  </si>
-  <si>
-    <t>1050.62</t>
-  </si>
-  <si>
-    <t>5341597-01</t>
-  </si>
-  <si>
-    <t>1235.47</t>
-  </si>
-  <si>
-    <t>100.50</t>
   </si>
   <si>
     <t>5506307-01</t>
@@ -2809,7 +2812,7 @@
         <v>21</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>46</v>
@@ -2874,13 +2877,13 @@
         <v>21</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>25</v>
@@ -2913,10 +2916,10 @@
         <v>88</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="Q18" s="1" t="s">
         <v>69</v>
@@ -2939,13 +2942,13 @@
         <v>21</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>25</v>
@@ -2978,10 +2981,10 @@
         <v>88</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Q19" s="1" t="s">
         <v>69</v>
@@ -3004,13 +3007,13 @@
         <v>21</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>25</v>
@@ -3043,10 +3046,10 @@
         <v>92</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q20" s="1" t="s">
         <v>69</v>
@@ -3069,13 +3072,13 @@
         <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>25</v>
@@ -3108,10 +3111,10 @@
         <v>92</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q21" s="1" t="s">
         <v>69</v>
@@ -3173,10 +3176,10 @@
         <v>92</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q22" s="1" t="s">
         <v>69</v>
@@ -3199,13 +3202,13 @@
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>25</v>
@@ -3238,10 +3241,10 @@
         <v>92</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q23" s="1" t="s">
         <v>69</v>
@@ -3264,13 +3267,13 @@
         <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>25</v>
@@ -3303,10 +3306,10 @@
         <v>92</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="Q24" s="1" t="s">
         <v>69</v>
@@ -3329,13 +3332,13 @@
         <v>21</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>25</v>
@@ -3368,10 +3371,10 @@
         <v>92</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q25" s="1" t="s">
         <v>69</v>
@@ -3394,13 +3397,13 @@
         <v>21</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>25</v>
@@ -3418,7 +3421,7 @@
         <v>29</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K26" s="1" t="n">
         <v>12</v>
@@ -3430,13 +3433,13 @@
         <v>31</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Q26" s="1" t="s">
         <v>69</v>
@@ -3459,13 +3462,13 @@
         <v>21</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>25</v>
@@ -3498,10 +3501,10 @@
         <v>92</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q27" s="1" t="s">
         <v>69</v>
@@ -3524,13 +3527,13 @@
         <v>21</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>25</v>
@@ -3548,7 +3551,7 @@
         <v>29</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K28" s="1" t="n">
         <v>13</v>
@@ -3560,13 +3563,13 @@
         <v>31</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q28" s="1" t="s">
         <v>69</v>
@@ -3589,13 +3592,13 @@
         <v>21</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>25</v>
@@ -3613,7 +3616,7 @@
         <v>29</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K29" s="1" t="n">
         <v>13</v>
@@ -3625,13 +3628,13 @@
         <v>31</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q29" s="1" t="s">
         <v>69</v>
@@ -3654,13 +3657,13 @@
         <v>21</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>25</v>
@@ -3678,7 +3681,7 @@
         <v>29</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K30" s="1" t="n">
         <v>13</v>
@@ -3690,13 +3693,13 @@
         <v>31</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="Q30" s="1" t="s">
         <v>69</v>
@@ -3719,13 +3722,13 @@
         <v>21</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>40</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>25</v>
@@ -3758,10 +3761,10 @@
         <v>43</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="Q31" s="1" t="s">
         <v>69</v>
@@ -3784,13 +3787,13 @@
         <v>21</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>25</v>
@@ -3808,7 +3811,7 @@
         <v>29</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K32" s="1" t="n">
         <v>14</v>
@@ -3820,13 +3823,13 @@
         <v>31</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q32" s="1" t="s">
         <v>69</v>
@@ -3849,13 +3852,13 @@
         <v>21</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>25</v>
@@ -3873,7 +3876,7 @@
         <v>29</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K33" s="1" t="n">
         <v>14</v>
@@ -3885,13 +3888,13 @@
         <v>31</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="Q33" s="1" t="s">
         <v>69</v>
@@ -3914,13 +3917,13 @@
         <v>21</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>25</v>
@@ -3938,7 +3941,7 @@
         <v>29</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K34" s="1" t="n">
         <v>15</v>
@@ -3950,13 +3953,13 @@
         <v>31</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="P34" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="Q34" s="1" t="s">
         <v>69</v>
@@ -3979,13 +3982,13 @@
         <v>21</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>25</v>
@@ -4003,7 +4006,7 @@
         <v>29</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K35" s="1" t="n">
         <v>16</v>
@@ -4015,13 +4018,13 @@
         <v>31</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q35" s="1" t="s">
         <v>69</v>
@@ -4044,13 +4047,13 @@
         <v>21</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>25</v>
@@ -4068,7 +4071,7 @@
         <v>29</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K36" s="1" t="n">
         <v>16</v>
@@ -4080,13 +4083,13 @@
         <v>31</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Q36" s="1" t="s">
         <v>69</v>
@@ -4109,13 +4112,13 @@
         <v>21</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>25</v>
@@ -4133,7 +4136,7 @@
         <v>29</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K37" s="1" t="n">
         <v>16</v>
@@ -4145,13 +4148,13 @@
         <v>31</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="Q37" s="1" t="s">
         <v>69</v>
@@ -4174,13 +4177,13 @@
         <v>21</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>25</v>
@@ -4198,7 +4201,7 @@
         <v>29</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K38" s="1" t="n">
         <v>16</v>
@@ -4210,13 +4213,13 @@
         <v>31</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Q38" s="1" t="s">
         <v>69</v>
@@ -4239,13 +4242,13 @@
         <v>21</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>25</v>
@@ -4263,7 +4266,7 @@
         <v>29</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K39" s="1" t="n">
         <v>16</v>
@@ -4275,13 +4278,13 @@
         <v>31</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="Q39" s="1" t="s">
         <v>69</v>
@@ -4304,13 +4307,13 @@
         <v>21</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>25</v>
@@ -4343,10 +4346,10 @@
         <v>92</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="Q40" s="1" t="s">
         <v>69</v>
@@ -4369,13 +4372,13 @@
         <v>21</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>25</v>
@@ -4408,10 +4411,10 @@
         <v>92</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q41" s="1" t="s">
         <v>69</v>
@@ -4434,13 +4437,13 @@
         <v>21</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>25</v>
@@ -4473,10 +4476,10 @@
         <v>92</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Q42" s="1" t="s">
         <v>69</v>
@@ -4499,13 +4502,13 @@
         <v>21</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>25</v>
@@ -4523,7 +4526,7 @@
         <v>29</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K43" s="1" t="n">
         <v>20</v>
@@ -4535,13 +4538,13 @@
         <v>31</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="Q43" s="1" t="s">
         <v>69</v>
@@ -4564,13 +4567,13 @@
         <v>21</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>25</v>
@@ -4588,7 +4591,7 @@
         <v>29</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K44" s="1" t="n">
         <v>21</v>
@@ -4600,13 +4603,13 @@
         <v>31</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O44" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Q44" s="1" t="s">
         <v>69</v>
@@ -4629,13 +4632,13 @@
         <v>21</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>25</v>
@@ -4653,7 +4656,7 @@
         <v>29</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K45" s="1" t="n">
         <v>24</v>
@@ -4665,13 +4668,13 @@
         <v>31</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O45" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Q45" s="1" t="s">
         <v>69</v>
@@ -4694,13 +4697,13 @@
         <v>21</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>25</v>
@@ -4718,7 +4721,7 @@
         <v>29</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K46" s="1" t="n">
         <v>27</v>
@@ -4730,13 +4733,13 @@
         <v>31</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Q46" s="1" t="s">
         <v>69</v>
@@ -4759,22 +4762,22 @@
         <v>21</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H47" s="1" t="s">
         <v>28</v>
@@ -4786,7 +4789,7 @@
         <v>30</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L47" s="1" t="n">
         <v>1</v>
@@ -4798,10 +4801,10 @@
         <v>92</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="Q47" s="1" t="s">
         <v>69</v>
@@ -4824,22 +4827,22 @@
         <v>21</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H48" s="1" t="s">
         <v>28</v>
@@ -4851,7 +4854,7 @@
         <v>30</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L48" s="1" t="n">
         <v>1</v>
@@ -4863,10 +4866,10 @@
         <v>92</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="Q48" s="1" t="s">
         <v>69</v>
@@ -4889,22 +4892,22 @@
         <v>21</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H49" s="1" t="s">
         <v>28</v>
@@ -4916,7 +4919,7 @@
         <v>30</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L49" s="1" t="n">
         <v>1</v>
@@ -4928,10 +4931,10 @@
         <v>92</v>
       </c>
       <c r="O49" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="Q49" s="1" t="s">
         <v>69</v>
@@ -4954,22 +4957,22 @@
         <v>21</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H50" s="1" t="s">
         <v>28</v>
@@ -4981,7 +4984,7 @@
         <v>30</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L50" s="1" t="n">
         <v>1</v>
@@ -4993,10 +4996,10 @@
         <v>92</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P50" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="Q50" s="1" t="s">
         <v>69</v>
@@ -5019,13 +5022,13 @@
         <v>21</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>25</v>
@@ -5034,10 +5037,10 @@
         <v>26</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>29</v>
@@ -5055,16 +5058,16 @@
         <v>31</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="O51" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="P51" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="R51" s="1" t="s">
         <v>36</v>
@@ -5084,13 +5087,13 @@
         <v>21</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>25</v>
@@ -5108,7 +5111,7 @@
         <v>29</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K52" s="1" t="n">
         <v>8</v>
@@ -5123,13 +5126,13 @@
         <v>88</v>
       </c>
       <c r="O52" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="P52" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="R52" s="1" t="s">
         <v>36</v>
@@ -5149,13 +5152,13 @@
         <v>21</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>25</v>
@@ -5173,7 +5176,7 @@
         <v>29</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K53" s="1" t="n">
         <v>12</v>
@@ -5185,16 +5188,16 @@
         <v>31</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="O53" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P53" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q53" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="R53" s="1" t="s">
         <v>36</v>
@@ -5211,13 +5214,13 @@
         <v>21</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>25</v>
@@ -5250,13 +5253,13 @@
         <v>49</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="P54" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="Q54" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="R54" s="1" t="s">
         <v>36</v>
@@ -5276,13 +5279,13 @@
         <v>21</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>25</v>
@@ -5315,13 +5318,13 @@
         <v>49</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P55" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="Q55" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="R55" s="1" t="s">
         <v>36</v>
@@ -5341,13 +5344,13 @@
         <v>21</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>25</v>
@@ -5380,13 +5383,13 @@
         <v>49</v>
       </c>
       <c r="O56" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="P56" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="Q56" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="R56" s="1" t="s">
         <v>36</v>
@@ -5406,13 +5409,13 @@
         <v>21</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>25</v>
@@ -5445,13 +5448,13 @@
         <v>49</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="P57" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="Q57" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="R57" s="1" t="s">
         <v>36</v>
@@ -5471,13 +5474,13 @@
         <v>21</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>25</v>
@@ -5495,7 +5498,7 @@
         <v>29</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K58" s="1" t="n">
         <v>21</v>
@@ -5507,16 +5510,16 @@
         <v>31</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O58" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="P58" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q58" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="R58" s="1" t="s">
         <v>36</v>
@@ -5536,13 +5539,13 @@
         <v>21</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>25</v>
@@ -5560,7 +5563,7 @@
         <v>29</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K59" s="1" t="n">
         <v>3</v>
@@ -5572,16 +5575,16 @@
         <v>31</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O59" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="P59" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q59" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R59" s="1" t="s">
         <v>36</v>
@@ -5601,13 +5604,13 @@
         <v>21</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>25</v>
@@ -5625,7 +5628,7 @@
         <v>29</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K60" s="1" t="n">
         <v>4</v>
@@ -5637,16 +5640,16 @@
         <v>31</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O60" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P60" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="Q60" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R60" s="1" t="s">
         <v>36</v>
@@ -5666,10 +5669,10 @@
         <v>21</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>24</v>
@@ -5702,16 +5705,16 @@
         <v>31</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="O61" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P61" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="Q61" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R61" s="1" t="s">
         <v>36</v>
@@ -5767,16 +5770,16 @@
         <v>31</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="O62" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P62" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="Q62" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R62" s="1" t="s">
         <v>36</v>
@@ -5796,13 +5799,13 @@
         <v>21</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>25</v>
@@ -5832,16 +5835,16 @@
         <v>31</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="O63" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="P63" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="Q63" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R63" s="1" t="s">
         <v>36</v>
@@ -5861,13 +5864,13 @@
         <v>21</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>25</v>
@@ -5885,7 +5888,7 @@
         <v>29</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K64" s="1" t="n">
         <v>13</v>
@@ -5897,16 +5900,16 @@
         <v>31</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="O64" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="P64" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q64" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R64" s="1" t="s">
         <v>36</v>
@@ -5926,31 +5929,31 @@
         <v>21</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K65" s="1" t="n">
         <v>22</v>
@@ -5962,16 +5965,16 @@
         <v>31</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="O65" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="P65" s="1" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q65" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R65" s="1" t="s">
         <v>36</v>
@@ -5988,13 +5991,13 @@
         <v>21</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>25</v>
@@ -6012,7 +6015,7 @@
         <v>29</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K66" s="1" t="n">
         <v>20</v>
@@ -6024,16 +6027,16 @@
         <v>31</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="O66" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="P66" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="R66" s="1" t="s">
         <v>36</v>
@@ -6053,13 +6056,13 @@
         <v>21</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>25</v>
@@ -6092,13 +6095,13 @@
         <v>88</v>
       </c>
       <c r="O67" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="P67" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q67" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="R67" s="1" t="s">
         <v>36</v>
@@ -6118,13 +6121,13 @@
         <v>21</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>25</v>
@@ -6142,7 +6145,7 @@
         <v>29</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K68" s="1" t="n">
         <v>3</v>
@@ -6154,16 +6157,16 @@
         <v>31</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="P68" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="Q68" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R68" s="1" t="s">
         <v>36</v>
@@ -6183,31 +6186,31 @@
         <v>21</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F69" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>29</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K69" s="1" t="n">
         <v>11</v>
@@ -6219,16 +6222,16 @@
         <v>31</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P69" s="1" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="Q69" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R69" s="1" t="s">
         <v>36</v>
@@ -6248,13 +6251,13 @@
         <v>21</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>25</v>
@@ -6272,7 +6275,7 @@
         <v>29</v>
       </c>
       <c r="J70" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K70" s="1" t="n">
         <v>19</v>
@@ -6284,16 +6287,16 @@
         <v>31</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="O70" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="P70" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="Q70" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R70" s="1" t="s">
         <v>36</v>
@@ -6313,13 +6316,13 @@
         <v>21</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>25</v>
@@ -6337,7 +6340,7 @@
         <v>29</v>
       </c>
       <c r="J71" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K71" s="1" t="n">
         <v>20</v>
@@ -6349,16 +6352,16 @@
         <v>31</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="O71" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="P71" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="Q71" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R71" s="1" t="s">
         <v>36</v>
@@ -6378,13 +6381,13 @@
         <v>21</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>25</v>
@@ -6402,7 +6405,7 @@
         <v>29</v>
       </c>
       <c r="J72" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K72" s="1" t="n">
         <v>21</v>
@@ -6414,16 +6417,16 @@
         <v>31</v>
       </c>
       <c r="N72" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="O72" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="P72" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="Q72" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R72" s="1" t="s">
         <v>36</v>
@@ -6443,13 +6446,13 @@
         <v>21</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>25</v>
@@ -6467,7 +6470,7 @@
         <v>29</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K73" s="1" t="n">
         <v>21</v>
@@ -6479,16 +6482,16 @@
         <v>31</v>
       </c>
       <c r="N73" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="O73" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="P73" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="Q73" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R73" s="1" t="s">
         <v>36</v>
@@ -6508,13 +6511,13 @@
         <v>21</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>25</v>
@@ -6532,7 +6535,7 @@
         <v>29</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K74" s="1" t="n">
         <v>21</v>
@@ -6544,16 +6547,16 @@
         <v>31</v>
       </c>
       <c r="N74" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="O74" s="1" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="P74" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="Q74" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="R74" s="1" t="s">
         <v>36</v>
@@ -6573,13 +6576,13 @@
         <v>21</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E75" s="1" t="s">
         <v>25</v>
@@ -6609,16 +6612,16 @@
         <v>31</v>
       </c>
       <c r="N75" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="O75" s="1" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="P75" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="Q75" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="R75" s="1" t="s">
         <v>36</v>
@@ -6638,13 +6641,13 @@
         <v>21</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>25</v>
@@ -6674,16 +6677,16 @@
         <v>31</v>
       </c>
       <c r="N76" s="1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="O76" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="P76" s="1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="Q76" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="R76" s="1" t="s">
         <v>36</v>
@@ -6703,13 +6706,13 @@
         <v>21</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>25</v>
@@ -6739,16 +6742,16 @@
         <v>31</v>
       </c>
       <c r="N77" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O77" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="P77" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="Q77" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="R77" s="1" t="s">
         <v>36</v>
@@ -6768,13 +6771,13 @@
         <v>21</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>25</v>
@@ -6792,7 +6795,7 @@
         <v>29</v>
       </c>
       <c r="J78" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K78" s="1" t="n">
         <v>15</v>
@@ -6804,16 +6807,16 @@
         <v>31</v>
       </c>
       <c r="N78" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="O78" s="1" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="P78" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="Q78" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="R78" s="1" t="s">
         <v>36</v>
@@ -6833,31 +6836,31 @@
         <v>21</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F79" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I79" s="1" t="s">
         <v>29</v>
       </c>
       <c r="J79" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K79" s="1" t="n">
         <v>11</v>
@@ -6869,16 +6872,16 @@
         <v>31</v>
       </c>
       <c r="N79" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O79" s="1" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="P79" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="Q79" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R79" s="1" t="s">
         <v>36</v>
@@ -6898,13 +6901,13 @@
         <v>21</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>25</v>
@@ -6922,7 +6925,7 @@
         <v>29</v>
       </c>
       <c r="J80" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K80" s="1" t="n">
         <v>13</v>
@@ -6934,16 +6937,16 @@
         <v>31</v>
       </c>
       <c r="N80" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="O80" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="P80" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="Q80" s="1" t="s">
         <v>370</v>
-      </c>
-      <c r="O80" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="P80" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="Q80" s="1" t="s">
-        <v>369</v>
       </c>
       <c r="R80" s="1" t="s">
         <v>36</v>
@@ -6963,13 +6966,13 @@
         <v>21</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E81" s="1" t="s">
         <v>25</v>
@@ -6987,7 +6990,7 @@
         <v>29</v>
       </c>
       <c r="J81" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K81" s="1" t="n">
         <v>13</v>
@@ -6999,16 +7002,16 @@
         <v>31</v>
       </c>
       <c r="N81" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O81" s="1" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="P81" s="1" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="Q81" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R81" s="1" t="s">
         <v>36</v>
@@ -7028,13 +7031,13 @@
         <v>21</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>25</v>
@@ -7052,7 +7055,7 @@
         <v>29</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K82" s="1" t="n">
         <v>13</v>
@@ -7064,16 +7067,16 @@
         <v>31</v>
       </c>
       <c r="N82" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O82" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="P82" s="1" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="Q82" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R82" s="1" t="s">
         <v>36</v>
@@ -7093,13 +7096,13 @@
         <v>21</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E83" s="1" t="s">
         <v>25</v>
@@ -7117,7 +7120,7 @@
         <v>29</v>
       </c>
       <c r="J83" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K83" s="1" t="n">
         <v>13</v>
@@ -7129,16 +7132,16 @@
         <v>31</v>
       </c>
       <c r="N83" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O83" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="P83" s="1" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="Q83" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R83" s="1" t="s">
         <v>36</v>
@@ -7158,13 +7161,13 @@
         <v>21</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>40</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>25</v>
@@ -7194,16 +7197,16 @@
         <v>31</v>
       </c>
       <c r="N84" s="1" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="O84" s="1" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P84" s="1" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="Q84" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R84" s="1" t="s">
         <v>36</v>
@@ -7223,13 +7226,13 @@
         <v>21</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E85" s="1" t="s">
         <v>25</v>
@@ -7247,7 +7250,7 @@
         <v>29</v>
       </c>
       <c r="J85" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K85" s="1" t="n">
         <v>14</v>
@@ -7259,16 +7262,16 @@
         <v>31</v>
       </c>
       <c r="N85" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O85" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="P85" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="Q85" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R85" s="1" t="s">
         <v>36</v>
@@ -7288,13 +7291,13 @@
         <v>21</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E86" s="1" t="s">
         <v>25</v>
@@ -7312,7 +7315,7 @@
         <v>29</v>
       </c>
       <c r="J86" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K86" s="1" t="n">
         <v>14</v>
@@ -7324,16 +7327,16 @@
         <v>31</v>
       </c>
       <c r="N86" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="O86" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="P86" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="Q86" s="1" t="s">
         <v>370</v>
-      </c>
-      <c r="O86" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="P86" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="Q86" s="1" t="s">
-        <v>369</v>
       </c>
       <c r="R86" s="1" t="s">
         <v>36</v>
@@ -7353,13 +7356,13 @@
         <v>21</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E87" s="1" t="s">
         <v>25</v>
@@ -7377,7 +7380,7 @@
         <v>29</v>
       </c>
       <c r="J87" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K87" s="1" t="n">
         <v>14</v>
@@ -7389,16 +7392,16 @@
         <v>31</v>
       </c>
       <c r="N87" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="O87" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="P87" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="Q87" s="1" t="s">
         <v>370</v>
-      </c>
-      <c r="O87" s="1" t="s">
-        <v>400</v>
-      </c>
-      <c r="P87" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="Q87" s="1" t="s">
-        <v>369</v>
       </c>
       <c r="R87" s="1" t="s">
         <v>36</v>
@@ -7418,13 +7421,13 @@
         <v>21</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>25</v>
@@ -7442,7 +7445,7 @@
         <v>29</v>
       </c>
       <c r="J88" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K88" s="1" t="n">
         <v>14</v>
@@ -7454,16 +7457,16 @@
         <v>31</v>
       </c>
       <c r="N88" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O88" s="1" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="P88" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="Q88" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R88" s="1" t="s">
         <v>36</v>
@@ -7483,13 +7486,13 @@
         <v>21</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E89" s="1" t="s">
         <v>25</v>
@@ -7507,7 +7510,7 @@
         <v>29</v>
       </c>
       <c r="J89" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K89" s="1" t="n">
         <v>14</v>
@@ -7519,16 +7522,16 @@
         <v>31</v>
       </c>
       <c r="N89" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O89" s="1" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="P89" s="1" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="Q89" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R89" s="1" t="s">
         <v>36</v>
@@ -7548,13 +7551,13 @@
         <v>21</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E90" s="1" t="s">
         <v>25</v>
@@ -7572,7 +7575,7 @@
         <v>29</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K90" s="1" t="n">
         <v>14</v>
@@ -7584,16 +7587,16 @@
         <v>31</v>
       </c>
       <c r="N90" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O90" s="1" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="P90" s="1" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="Q90" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R90" s="1" t="s">
         <v>36</v>
@@ -7613,13 +7616,13 @@
         <v>21</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>25</v>
@@ -7637,7 +7640,7 @@
         <v>29</v>
       </c>
       <c r="J91" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K91" s="1" t="n">
         <v>14</v>
@@ -7649,16 +7652,16 @@
         <v>31</v>
       </c>
       <c r="N91" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O91" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P91" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="Q91" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R91" s="1" t="s">
         <v>36</v>
@@ -7678,13 +7681,13 @@
         <v>21</v>
       </c>
       <c r="B92" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="D92" s="1" t="s">
         <v>420</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>419</v>
       </c>
       <c r="E92" s="1" t="s">
         <v>25</v>
@@ -7702,7 +7705,7 @@
         <v>29</v>
       </c>
       <c r="J92" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K92" s="1" t="n">
         <v>14</v>
@@ -7714,16 +7717,16 @@
         <v>31</v>
       </c>
       <c r="N92" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O92" s="1" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="P92" s="1" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="Q92" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R92" s="1" t="s">
         <v>36</v>
@@ -7743,13 +7746,13 @@
         <v>21</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>25</v>
@@ -7767,7 +7770,7 @@
         <v>29</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K93" s="1" t="n">
         <v>14</v>
@@ -7779,16 +7782,16 @@
         <v>31</v>
       </c>
       <c r="N93" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O93" s="1" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="P93" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q93" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R93" s="1" t="s">
         <v>36</v>
@@ -7808,13 +7811,13 @@
         <v>21</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E94" s="1" t="s">
         <v>25</v>
@@ -7832,7 +7835,7 @@
         <v>29</v>
       </c>
       <c r="J94" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K94" s="1" t="n">
         <v>14</v>
@@ -7844,16 +7847,16 @@
         <v>31</v>
       </c>
       <c r="N94" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O94" s="1" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="P94" s="1" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="Q94" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R94" s="1" t="s">
         <v>36</v>
@@ -7873,13 +7876,13 @@
         <v>21</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E95" s="1" t="s">
         <v>25</v>
@@ -7897,7 +7900,7 @@
         <v>29</v>
       </c>
       <c r="J95" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K95" s="1" t="n">
         <v>14</v>
@@ -7909,16 +7912,16 @@
         <v>31</v>
       </c>
       <c r="N95" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O95" s="1" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="P95" s="1" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Q95" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R95" s="1" t="s">
         <v>36</v>
@@ -7938,13 +7941,13 @@
         <v>21</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E96" s="1" t="s">
         <v>25</v>
@@ -7962,7 +7965,7 @@
         <v>29</v>
       </c>
       <c r="J96" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K96" s="1" t="n">
         <v>14</v>
@@ -7974,16 +7977,16 @@
         <v>31</v>
       </c>
       <c r="N96" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O96" s="1" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="P96" s="1" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="Q96" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R96" s="1" t="s">
         <v>36</v>
@@ -8003,13 +8006,13 @@
         <v>21</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E97" s="1" t="s">
         <v>25</v>
@@ -8027,7 +8030,7 @@
         <v>29</v>
       </c>
       <c r="J97" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K97" s="1" t="n">
         <v>15</v>
@@ -8039,16 +8042,16 @@
         <v>31</v>
       </c>
       <c r="N97" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O97" s="1" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="P97" s="1" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="Q97" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R97" s="1" t="s">
         <v>36</v>
@@ -8068,13 +8071,13 @@
         <v>21</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E98" s="1" t="s">
         <v>25</v>
@@ -8092,7 +8095,7 @@
         <v>29</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K98" s="1" t="n">
         <v>15</v>
@@ -8104,16 +8107,16 @@
         <v>31</v>
       </c>
       <c r="N98" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O98" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P98" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="Q98" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R98" s="1" t="s">
         <v>36</v>
@@ -8133,13 +8136,13 @@
         <v>21</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E99" s="1" t="s">
         <v>25</v>
@@ -8157,7 +8160,7 @@
         <v>29</v>
       </c>
       <c r="J99" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K99" s="1" t="n">
         <v>15</v>
@@ -8169,16 +8172,16 @@
         <v>31</v>
       </c>
       <c r="N99" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O99" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P99" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="Q99" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R99" s="1" t="s">
         <v>36</v>
@@ -8198,13 +8201,13 @@
         <v>21</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E100" s="1" t="s">
         <v>25</v>
@@ -8222,7 +8225,7 @@
         <v>29</v>
       </c>
       <c r="J100" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K100" s="1" t="n">
         <v>15</v>
@@ -8234,16 +8237,16 @@
         <v>31</v>
       </c>
       <c r="N100" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O100" s="1" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="P100" s="1" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="Q100" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R100" s="1" t="s">
         <v>36</v>
@@ -8263,13 +8266,13 @@
         <v>21</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E101" s="1" t="s">
         <v>25</v>
@@ -8287,7 +8290,7 @@
         <v>29</v>
       </c>
       <c r="J101" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K101" s="1" t="n">
         <v>15</v>
@@ -8299,16 +8302,16 @@
         <v>31</v>
       </c>
       <c r="N101" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O101" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P101" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="Q101" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R101" s="1" t="s">
         <v>36</v>
@@ -8328,13 +8331,13 @@
         <v>21</v>
       </c>
       <c r="B102" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="D102" s="1" t="s">
         <v>457</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="D102" s="1" t="s">
-        <v>456</v>
       </c>
       <c r="E102" s="1" t="s">
         <v>25</v>
@@ -8352,7 +8355,7 @@
         <v>29</v>
       </c>
       <c r="J102" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K102" s="1" t="n">
         <v>15</v>
@@ -8364,16 +8367,16 @@
         <v>31</v>
       </c>
       <c r="N102" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="O102" s="1" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="P102" s="1" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="Q102" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R102" s="1" t="s">
         <v>36</v>
@@ -8393,13 +8396,13 @@
         <v>21</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E103" s="1" t="s">
         <v>25</v>
@@ -8417,7 +8420,7 @@
         <v>29</v>
       </c>
       <c r="J103" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K103" s="1" t="n">
         <v>15</v>
@@ -8429,16 +8432,16 @@
         <v>31</v>
       </c>
       <c r="N103" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O103" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="P103" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="Q103" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R103" s="1" t="s">
         <v>36</v>
@@ -8458,13 +8461,13 @@
         <v>21</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E104" s="1" t="s">
         <v>25</v>
@@ -8482,7 +8485,7 @@
         <v>29</v>
       </c>
       <c r="J104" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K104" s="1" t="n">
         <v>15</v>
@@ -8494,16 +8497,16 @@
         <v>31</v>
       </c>
       <c r="N104" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="O104" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="P104" s="1" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="Q104" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R104" s="1" t="s">
         <v>36</v>
@@ -8523,13 +8526,13 @@
         <v>21</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E105" s="1" t="s">
         <v>25</v>
@@ -8547,7 +8550,7 @@
         <v>29</v>
       </c>
       <c r="J105" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K105" s="1" t="n">
         <v>15</v>
@@ -8562,13 +8565,13 @@
         <v>92</v>
       </c>
       <c r="O105" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="P105" s="1" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="Q105" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R105" s="1" t="s">
         <v>36</v>
@@ -8588,13 +8591,13 @@
         <v>21</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E106" s="1" t="s">
         <v>25</v>
@@ -8612,7 +8615,7 @@
         <v>29</v>
       </c>
       <c r="J106" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K106" s="1" t="n">
         <v>16</v>
@@ -8624,16 +8627,16 @@
         <v>31</v>
       </c>
       <c r="N106" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="O106" s="1" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P106" s="1" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="Q106" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R106" s="1" t="s">
         <v>36</v>
@@ -8653,13 +8656,13 @@
         <v>21</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E107" s="1" t="s">
         <v>25</v>
@@ -8677,7 +8680,7 @@
         <v>29</v>
       </c>
       <c r="J107" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K107" s="1" t="n">
         <v>16</v>
@@ -8692,13 +8695,13 @@
         <v>43</v>
       </c>
       <c r="O107" s="1" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="P107" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="Q107" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R107" s="1" t="s">
         <v>36</v>
@@ -8718,13 +8721,13 @@
         <v>21</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E108" s="1" t="s">
         <v>25</v>
@@ -8742,7 +8745,7 @@
         <v>29</v>
       </c>
       <c r="J108" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K108" s="1" t="n">
         <v>16</v>
@@ -8754,16 +8757,16 @@
         <v>31</v>
       </c>
       <c r="N108" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O108" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P108" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="Q108" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R108" s="1" t="s">
         <v>36</v>
@@ -8783,13 +8786,13 @@
         <v>21</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E109" s="1" t="s">
         <v>25</v>
@@ -8819,16 +8822,16 @@
         <v>31</v>
       </c>
       <c r="N109" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O109" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="P109" s="1" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="Q109" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R109" s="1" t="s">
         <v>36</v>
@@ -8848,13 +8851,13 @@
         <v>21</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E110" s="1" t="s">
         <v>25</v>
@@ -8884,16 +8887,16 @@
         <v>31</v>
       </c>
       <c r="N110" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O110" s="1" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="P110" s="1" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="Q110" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R110" s="1" t="s">
         <v>36</v>
@@ -8949,16 +8952,16 @@
         <v>31</v>
       </c>
       <c r="N111" s="1" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="O111" s="1" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="P111" s="1" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="Q111" s="1" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="R111" s="1" t="s">
         <v>36</v>
@@ -8978,13 +8981,13 @@
         <v>21</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E112" s="1" t="s">
         <v>25</v>
@@ -9014,16 +9017,16 @@
         <v>31</v>
       </c>
       <c r="N112" s="1" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="O112" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="P112" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="Q112" s="1" t="s">
         <v>491</v>
-      </c>
-      <c r="Q112" s="1" t="s">
-        <v>490</v>
       </c>
       <c r="R112" s="1" t="s">
         <v>36</v>
@@ -9043,31 +9046,31 @@
         <v>21</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G113" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H113" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I113" s="1" t="s">
         <v>29</v>
       </c>
       <c r="J113" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K113" s="1" t="n">
         <v>11</v>
@@ -9079,16 +9082,16 @@
         <v>31</v>
       </c>
       <c r="N113" s="1" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="O113" s="1" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="P113" s="1" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="Q113" s="1" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="R113" s="1" t="s">
         <v>36</v>
@@ -9108,13 +9111,13 @@
         <v>21</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E114" s="1" t="s">
         <v>25</v>
@@ -9132,7 +9135,7 @@
         <v>29</v>
       </c>
       <c r="J114" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K114" s="1" t="n">
         <v>13</v>
@@ -9144,16 +9147,16 @@
         <v>31</v>
       </c>
       <c r="N114" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="O114" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="P114" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="Q114" s="1" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="R114" s="1" t="s">
         <v>36</v>
@@ -9173,13 +9176,13 @@
         <v>21</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E115" s="1" t="s">
         <v>25</v>
@@ -9197,7 +9200,7 @@
         <v>29</v>
       </c>
       <c r="J115" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K115" s="1" t="n">
         <v>15</v>
@@ -9209,16 +9212,16 @@
         <v>31</v>
       </c>
       <c r="N115" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O115" s="1" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="P115" s="1" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="Q115" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="R115" s="1" t="s">
         <v>36</v>
@@ -9238,31 +9241,31 @@
         <v>21</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>26</v>
       </c>
       <c r="G116" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H116" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I116" s="1" t="s">
         <v>29</v>
       </c>
       <c r="J116" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K116" s="1" t="n">
         <v>11</v>
@@ -9274,16 +9277,16 @@
         <v>31</v>
       </c>
       <c r="N116" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="O116" s="1" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="P116" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="Q116" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="R116" s="1" t="s">
         <v>36</v>
@@ -9303,13 +9306,13 @@
         <v>21</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E117" s="1" t="s">
         <v>25</v>
@@ -9339,16 +9342,16 @@
         <v>31</v>
       </c>
       <c r="N117" s="1" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="O117" s="1" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="P117" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="Q117" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="R117" s="1" t="s">
         <v>36</v>
@@ -9368,13 +9371,13 @@
         <v>21</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E118" s="1" t="s">
         <v>25</v>
@@ -9392,7 +9395,7 @@
         <v>29</v>
       </c>
       <c r="J118" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K118" s="1" t="n">
         <v>15</v>
@@ -9404,16 +9407,16 @@
         <v>31</v>
       </c>
       <c r="N118" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="O118" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="P118" s="1" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="Q118" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="R118" s="1" t="s">
         <v>36</v>
@@ -9433,13 +9436,13 @@
         <v>21</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E119" s="1" t="s">
         <v>25</v>
@@ -9457,7 +9460,7 @@
         <v>29</v>
       </c>
       <c r="J119" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K119" s="1" t="n">
         <v>15</v>
@@ -9469,16 +9472,16 @@
         <v>31</v>
       </c>
       <c r="N119" s="1" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="O119" s="1" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="P119" s="1" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="Q119" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="R119" s="1" t="s">
         <v>36</v>
@@ -9498,13 +9501,13 @@
         <v>21</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E120" s="1" t="s">
         <v>25</v>
@@ -9522,7 +9525,7 @@
         <v>29</v>
       </c>
       <c r="J120" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K120" s="1" t="n">
         <v>15</v>
@@ -9534,16 +9537,16 @@
         <v>31</v>
       </c>
       <c r="N120" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="O120" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P120" s="1" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="Q120" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="R120" s="1" t="s">
         <v>36</v>
@@ -9563,13 +9566,13 @@
         <v>21</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E121" s="1" t="s">
         <v>25</v>
@@ -9587,7 +9590,7 @@
         <v>29</v>
       </c>
       <c r="J121" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K121" s="1" t="n">
         <v>15</v>
@@ -9599,16 +9602,16 @@
         <v>31</v>
       </c>
       <c r="N121" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="O121" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P121" s="1" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="Q121" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="R121" s="1" t="s">
         <v>36</v>
@@ -9628,13 +9631,13 @@
         <v>21</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E122" s="1" t="s">
         <v>25</v>
@@ -9664,16 +9667,16 @@
         <v>31</v>
       </c>
       <c r="N122" s="1" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="O122" s="1" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="P122" s="1" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="Q122" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="R122" s="1" t="s">
         <v>36</v>
@@ -9693,13 +9696,13 @@
         <v>21</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E123" s="1" t="s">
         <v>25</v>
@@ -9717,7 +9720,7 @@
         <v>29</v>
       </c>
       <c r="J123" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K123" s="1" t="n">
         <v>21</v>
@@ -9729,16 +9732,16 @@
         <v>31</v>
       </c>
       <c r="N123" s="1" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="O123" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P123" s="1" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="Q123" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="R123" s="1" t="s">
         <v>36</v>
@@ -9758,13 +9761,13 @@
         <v>21</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E124" s="1" t="s">
         <v>25</v>
@@ -9782,7 +9785,7 @@
         <v>29</v>
       </c>
       <c r="J124" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K124" s="1" t="n">
         <v>15</v>
@@ -9794,16 +9797,16 @@
         <v>31</v>
       </c>
       <c r="N124" s="1" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="O124" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="P124" s="1" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="Q124" s="1" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="R124" s="1" t="s">
         <v>36</v>
@@ -9823,13 +9826,13 @@
         <v>21</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E125" s="1" t="s">
         <v>25</v>
@@ -9847,7 +9850,7 @@
         <v>29</v>
       </c>
       <c r="J125" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K125" s="1" t="n">
         <v>16</v>
@@ -9859,16 +9862,16 @@
         <v>31</v>
       </c>
       <c r="N125" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="O125" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="P125" s="1" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="Q125" s="1" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="R125" s="1" t="s">
         <v>36</v>
@@ -9888,13 +9891,13 @@
         <v>21</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E126" s="1" t="s">
         <v>25</v>
@@ -9912,7 +9915,7 @@
         <v>29</v>
       </c>
       <c r="J126" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K126" s="1" t="n">
         <v>21</v>
@@ -9924,16 +9927,16 @@
         <v>31</v>
       </c>
       <c r="N126" s="1" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="O126" s="1" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="P126" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="Q126" s="1" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="R126" s="1" t="s">
         <v>36</v>

</xml_diff>